<commit_message>
Generator czasu pracy: strefa w 3 kolumnach (nazwa, godzina od, czas) x20
Zamiast tekstu w jednej komorce: Strefa N nazwa | godzina od | czas,
kolumny C..BJ. Godziny jako godzina Excela lub tekst G:MM. Task i import
potwierdzone na zywo w bazie Claude.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012jaRebrP6eX1f4AexjYN8z
</commit_message>
<xml_diff>
--- a/ImportyXML/Generator czasu pracy/Generator czasu pracy.xlsx
+++ b/ImportyXML/Generator czasu pracy/Generator czasu pracy.xlsx
@@ -28,22 +28,25 @@
     <t/>
   </si>
   <si>
-    <t>1. Wklej dane do arkusza „Dane” od wiersza 2: kolumna A = kod pracownika, B = data, C..V = Strefa 1..20.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   Jeden wiersz = jeden dzień jednego pracownika. Puste komórki stref są pomijane.</t>
-  </si>
-  <si>
-    <t>2. Komórka strefy = nazwa definicji strefy (dokładnie jak w enova), spacja, potem godziny:</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   • strefa z godziną od:   Nadgodziny 50% 16:00 2:00   (od 16:00, czas 2:00)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   • strefa z samym czasem: Dyżur domowy 4:00          (czas 4:00, bez godziny od)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   Ostatnia wartość to zawsze CZAS trwania (nie godzina do). Godziny w formacie G:MM.</t>
+    <t>1. Wklej dane do arkusza „Dane” od wiersza 2: kolumna A = kod pracownika, B = data,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   potem 20 stref po 3 kolumny (C..BJ): Strefa N nazwa | Strefa N godzina od | Strefa N czas.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Jeden wiersz = jeden dzień jednego pracownika. Strefy z trzema pustymi kolumnami są pomijane.</t>
+  </si>
+  <si>
+    <t>2. Nazwa = nazwa definicji strefy dokładnie jak w enova. Godzina od – tylko gdy strefa ma godziny</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   (zależnie od konfiguracji strefy), inaczej puste. Czas = czas trwania strefy (nie godzina do), wymagany.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Przykłady:  Nadgodziny 50% | 16:00 | 2:00     Dyżur domowy | (puste) | 4:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Godziny wpisuj jako G:MM (np. 16:00); godzina od może przekraczać 24:00 (do 47:59).</t>
   </si>
   <si>
     <t xml:space="preserve">   Strefy „Praca w normie” NIE wpisujemy – dopisuje ją automatycznie Task w enova na podstawie planu pracy.</t>
@@ -94,64 +97,184 @@
     <t>Data</t>
   </si>
   <si>
-    <t>Strefa 1</t>
-  </si>
-  <si>
-    <t>Strefa 2</t>
-  </si>
-  <si>
-    <t>Strefa 3</t>
-  </si>
-  <si>
-    <t>Strefa 4</t>
-  </si>
-  <si>
-    <t>Strefa 5</t>
-  </si>
-  <si>
-    <t>Strefa 6</t>
-  </si>
-  <si>
-    <t>Strefa 7</t>
-  </si>
-  <si>
-    <t>Strefa 8</t>
-  </si>
-  <si>
-    <t>Strefa 9</t>
-  </si>
-  <si>
-    <t>Strefa 10</t>
-  </si>
-  <si>
-    <t>Strefa 11</t>
-  </si>
-  <si>
-    <t>Strefa 12</t>
-  </si>
-  <si>
-    <t>Strefa 13</t>
-  </si>
-  <si>
-    <t>Strefa 14</t>
-  </si>
-  <si>
-    <t>Strefa 15</t>
-  </si>
-  <si>
-    <t>Strefa 16</t>
-  </si>
-  <si>
-    <t>Strefa 17</t>
-  </si>
-  <si>
-    <t>Strefa 18</t>
-  </si>
-  <si>
-    <t>Strefa 19</t>
-  </si>
-  <si>
-    <t>Strefa 20</t>
+    <t>Strefa 1 nazwa</t>
+  </si>
+  <si>
+    <t>Strefa 1 godzina od</t>
+  </si>
+  <si>
+    <t>Strefa 1 czas</t>
+  </si>
+  <si>
+    <t>Strefa 2 nazwa</t>
+  </si>
+  <si>
+    <t>Strefa 2 godzina od</t>
+  </si>
+  <si>
+    <t>Strefa 2 czas</t>
+  </si>
+  <si>
+    <t>Strefa 3 nazwa</t>
+  </si>
+  <si>
+    <t>Strefa 3 godzina od</t>
+  </si>
+  <si>
+    <t>Strefa 3 czas</t>
+  </si>
+  <si>
+    <t>Strefa 4 nazwa</t>
+  </si>
+  <si>
+    <t>Strefa 4 godzina od</t>
+  </si>
+  <si>
+    <t>Strefa 4 czas</t>
+  </si>
+  <si>
+    <t>Strefa 5 nazwa</t>
+  </si>
+  <si>
+    <t>Strefa 5 godzina od</t>
+  </si>
+  <si>
+    <t>Strefa 5 czas</t>
+  </si>
+  <si>
+    <t>Strefa 6 nazwa</t>
+  </si>
+  <si>
+    <t>Strefa 6 godzina od</t>
+  </si>
+  <si>
+    <t>Strefa 6 czas</t>
+  </si>
+  <si>
+    <t>Strefa 7 nazwa</t>
+  </si>
+  <si>
+    <t>Strefa 7 godzina od</t>
+  </si>
+  <si>
+    <t>Strefa 7 czas</t>
+  </si>
+  <si>
+    <t>Strefa 8 nazwa</t>
+  </si>
+  <si>
+    <t>Strefa 8 godzina od</t>
+  </si>
+  <si>
+    <t>Strefa 8 czas</t>
+  </si>
+  <si>
+    <t>Strefa 9 nazwa</t>
+  </si>
+  <si>
+    <t>Strefa 9 godzina od</t>
+  </si>
+  <si>
+    <t>Strefa 9 czas</t>
+  </si>
+  <si>
+    <t>Strefa 10 nazwa</t>
+  </si>
+  <si>
+    <t>Strefa 10 godzina od</t>
+  </si>
+  <si>
+    <t>Strefa 10 czas</t>
+  </si>
+  <si>
+    <t>Strefa 11 nazwa</t>
+  </si>
+  <si>
+    <t>Strefa 11 godzina od</t>
+  </si>
+  <si>
+    <t>Strefa 11 czas</t>
+  </si>
+  <si>
+    <t>Strefa 12 nazwa</t>
+  </si>
+  <si>
+    <t>Strefa 12 godzina od</t>
+  </si>
+  <si>
+    <t>Strefa 12 czas</t>
+  </si>
+  <si>
+    <t>Strefa 13 nazwa</t>
+  </si>
+  <si>
+    <t>Strefa 13 godzina od</t>
+  </si>
+  <si>
+    <t>Strefa 13 czas</t>
+  </si>
+  <si>
+    <t>Strefa 14 nazwa</t>
+  </si>
+  <si>
+    <t>Strefa 14 godzina od</t>
+  </si>
+  <si>
+    <t>Strefa 14 czas</t>
+  </si>
+  <si>
+    <t>Strefa 15 nazwa</t>
+  </si>
+  <si>
+    <t>Strefa 15 godzina od</t>
+  </si>
+  <si>
+    <t>Strefa 15 czas</t>
+  </si>
+  <si>
+    <t>Strefa 16 nazwa</t>
+  </si>
+  <si>
+    <t>Strefa 16 godzina od</t>
+  </si>
+  <si>
+    <t>Strefa 16 czas</t>
+  </si>
+  <si>
+    <t>Strefa 17 nazwa</t>
+  </si>
+  <si>
+    <t>Strefa 17 godzina od</t>
+  </si>
+  <si>
+    <t>Strefa 17 czas</t>
+  </si>
+  <si>
+    <t>Strefa 18 nazwa</t>
+  </si>
+  <si>
+    <t>Strefa 18 godzina od</t>
+  </si>
+  <si>
+    <t>Strefa 18 czas</t>
+  </si>
+  <si>
+    <t>Strefa 19 nazwa</t>
+  </si>
+  <si>
+    <t>Strefa 19 godzina od</t>
+  </si>
+  <si>
+    <t>Strefa 19 czas</t>
+  </si>
+  <si>
+    <t>Strefa 20 nazwa</t>
+  </si>
+  <si>
+    <t>Strefa 20 godzina od</t>
+  </si>
+  <si>
+    <t>Strefa 20 czas</t>
   </si>
   <si>
     <t>Wiersz</t>
@@ -167,8 +290,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+  <numFmts count="2">
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="164" formatCode="[h]:mm"/>
   </numFmts>
   <fonts count="2">
     <font>
@@ -198,13 +322,21 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -585,17 +717,22 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>1</v>
+        <v>15</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>15</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
         <v>16</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="s">
+        <v>17</v>
       </c>
     </row>
   </sheetData>
@@ -612,23 +749,23 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
   </sheetData>
@@ -641,94 +778,254 @@
   <cols>
     <col min="1" max="1" width="16.710938" style="2" customWidth="1"/>
     <col min="2" max="2" width="12.7109375" style="3" customWidth="1"/>
-    <col min="3" max="3" width="26.710938" style="2" customWidth="1"/>
-    <col min="4" max="4" width="26.710938" style="2" customWidth="1"/>
-    <col min="5" max="5" width="26.710938" style="2" customWidth="1"/>
-    <col min="6" max="6" width="26.710938" style="2" customWidth="1"/>
-    <col min="7" max="7" width="26.710938" style="2" customWidth="1"/>
-    <col min="8" max="8" width="26.710938" style="2" customWidth="1"/>
-    <col min="9" max="9" width="26.710938" style="2" customWidth="1"/>
-    <col min="10" max="10" width="26.710938" style="2" customWidth="1"/>
-    <col min="11" max="11" width="26.710938" style="2" customWidth="1"/>
-    <col min="12" max="12" width="26.710938" style="2" customWidth="1"/>
-    <col min="13" max="13" width="26.710938" style="2" customWidth="1"/>
-    <col min="14" max="14" width="26.710938" style="2" customWidth="1"/>
-    <col min="15" max="15" width="26.710938" style="2" customWidth="1"/>
-    <col min="16" max="16" width="26.710938" style="2" customWidth="1"/>
-    <col min="17" max="17" width="26.710938" style="2" customWidth="1"/>
-    <col min="18" max="18" width="26.710938" style="2" customWidth="1"/>
-    <col min="19" max="19" width="26.710938" style="2" customWidth="1"/>
-    <col min="20" max="20" width="26.710938" style="2" customWidth="1"/>
-    <col min="21" max="21" width="26.710938" style="2" customWidth="1"/>
-    <col min="22" max="22" width="26.710938" style="2" customWidth="1"/>
+    <col min="3" max="3" width="24.710938" style="2" customWidth="1"/>
+    <col min="4" max="4" width="10.7109375" style="4" customWidth="1"/>
+    <col min="5" max="5" width="10.7109375" style="4" customWidth="1"/>
+    <col min="6" max="6" width="24.710938" style="2" customWidth="1"/>
+    <col min="7" max="7" width="10.7109375" style="4" customWidth="1"/>
+    <col min="8" max="8" width="10.7109375" style="4" customWidth="1"/>
+    <col min="9" max="9" width="24.710938" style="2" customWidth="1"/>
+    <col min="10" max="10" width="10.7109375" style="4" customWidth="1"/>
+    <col min="11" max="11" width="10.7109375" style="4" customWidth="1"/>
+    <col min="12" max="12" width="24.710938" style="2" customWidth="1"/>
+    <col min="13" max="13" width="10.7109375" style="4" customWidth="1"/>
+    <col min="14" max="14" width="10.7109375" style="4" customWidth="1"/>
+    <col min="15" max="15" width="24.710938" style="2" customWidth="1"/>
+    <col min="16" max="16" width="10.7109375" style="4" customWidth="1"/>
+    <col min="17" max="17" width="10.7109375" style="4" customWidth="1"/>
+    <col min="18" max="18" width="24.710938" style="2" customWidth="1"/>
+    <col min="19" max="19" width="10.7109375" style="4" customWidth="1"/>
+    <col min="20" max="20" width="10.7109375" style="4" customWidth="1"/>
+    <col min="21" max="21" width="24.710938" style="2" customWidth="1"/>
+    <col min="22" max="22" width="10.7109375" style="4" customWidth="1"/>
+    <col min="23" max="23" width="10.7109375" style="4" customWidth="1"/>
+    <col min="24" max="24" width="24.710938" style="2" customWidth="1"/>
+    <col min="25" max="25" width="10.7109375" style="4" customWidth="1"/>
+    <col min="26" max="26" width="10.7109375" style="4" customWidth="1"/>
+    <col min="27" max="27" width="24.710938" style="2" customWidth="1"/>
+    <col min="28" max="28" width="10.7109375" style="4" customWidth="1"/>
+    <col min="29" max="29" width="10.7109375" style="4" customWidth="1"/>
+    <col min="30" max="30" width="24.710938" style="2" customWidth="1"/>
+    <col min="31" max="31" width="10.7109375" style="4" customWidth="1"/>
+    <col min="32" max="32" width="10.7109375" style="4" customWidth="1"/>
+    <col min="33" max="33" width="24.710938" style="2" customWidth="1"/>
+    <col min="34" max="34" width="10.7109375" style="4" customWidth="1"/>
+    <col min="35" max="35" width="10.7109375" style="4" customWidth="1"/>
+    <col min="36" max="36" width="24.710938" style="2" customWidth="1"/>
+    <col min="37" max="37" width="10.7109375" style="4" customWidth="1"/>
+    <col min="38" max="38" width="10.7109375" style="4" customWidth="1"/>
+    <col min="39" max="39" width="24.710938" style="2" customWidth="1"/>
+    <col min="40" max="40" width="10.7109375" style="4" customWidth="1"/>
+    <col min="41" max="41" width="10.7109375" style="4" customWidth="1"/>
+    <col min="42" max="42" width="24.710938" style="2" customWidth="1"/>
+    <col min="43" max="43" width="10.7109375" style="4" customWidth="1"/>
+    <col min="44" max="44" width="10.7109375" style="4" customWidth="1"/>
+    <col min="45" max="45" width="24.710938" style="2" customWidth="1"/>
+    <col min="46" max="46" width="10.7109375" style="4" customWidth="1"/>
+    <col min="47" max="47" width="10.7109375" style="4" customWidth="1"/>
+    <col min="48" max="48" width="24.710938" style="2" customWidth="1"/>
+    <col min="49" max="49" width="10.7109375" style="4" customWidth="1"/>
+    <col min="50" max="50" width="10.7109375" style="4" customWidth="1"/>
+    <col min="51" max="51" width="24.710938" style="2" customWidth="1"/>
+    <col min="52" max="52" width="10.7109375" style="4" customWidth="1"/>
+    <col min="53" max="53" width="10.7109375" style="4" customWidth="1"/>
+    <col min="54" max="54" width="24.710938" style="2" customWidth="1"/>
+    <col min="55" max="55" width="10.7109375" style="4" customWidth="1"/>
+    <col min="56" max="56" width="10.7109375" style="4" customWidth="1"/>
+    <col min="57" max="57" width="24.710938" style="2" customWidth="1"/>
+    <col min="58" max="58" width="10.7109375" style="4" customWidth="1"/>
+    <col min="59" max="59" width="10.7109375" style="4" customWidth="1"/>
+    <col min="60" max="60" width="24.710938" style="2" customWidth="1"/>
+    <col min="61" max="61" width="10.7109375" style="4" customWidth="1"/>
+    <col min="62" max="62" width="10.7109375" style="4" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="B1" s="5" t="s">
+    <row r="1" ht="30">
+      <c r="A1" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="B1" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="C1" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="D1" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="E1" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="F1" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="G1" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="H1" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="J1" s="4" t="s">
+      <c r="I1" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="K1" s="4" t="s">
+      <c r="J1" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="L1" s="4" t="s">
+      <c r="K1" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="M1" s="4" t="s">
+      <c r="L1" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="N1" s="4" t="s">
+      <c r="M1" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="O1" s="4" t="s">
+      <c r="N1" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="P1" s="4" t="s">
+      <c r="O1" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="Q1" s="4" t="s">
+      <c r="P1" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="R1" s="4" t="s">
+      <c r="Q1" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="S1" s="4" t="s">
+      <c r="R1" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="T1" s="4" t="s">
+      <c r="S1" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="U1" s="4" t="s">
+      <c r="T1" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="V1" s="4" t="s">
+      <c r="U1" s="5" t="s">
         <v>43</v>
+      </c>
+      <c r="V1" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="W1" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="X1" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="Y1" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="Z1" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="AA1" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="AB1" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="AC1" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="AD1" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="AE1" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="AF1" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="AG1" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="AH1" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="AI1" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="AJ1" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="AK1" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="AL1" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AM1" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="AN1" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="AO1" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="AP1" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="AQ1" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="AR1" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="AS1" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="AT1" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="AU1" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="AV1" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="AW1" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="AX1" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="AY1" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="AZ1" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="BA1" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="BB1" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="BC1" s="7" t="s">
+        <v>77</v>
+      </c>
+      <c r="BD1" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="BE1" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="BF1" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="BG1" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="BH1" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="BI1" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="BJ1" s="7" t="s">
+        <v>84</v>
       </c>
     </row>
   </sheetData>
@@ -747,16 +1044,16 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>44</v>
+        <v>85</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>45</v>
+        <v>86</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>46</v>
+        <v>87</v>
       </c>
     </row>
   </sheetData>

</xml_diff>